<commit_message>
cambio de imágenes y de archivo
</commit_message>
<xml_diff>
--- a/Dashboard_financiero_Excel.xlsx
+++ b/Dashboard_financiero_Excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sandr\OneDrive\Documentos\GitHub\Dashboard-financiero-Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05020C27-0A79-4DBD-8F3C-44D5323C3BA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D85E958F-D14B-401F-A884-E596300CA0BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="816" activeTab="1" xr2:uid="{92CC657A-38E7-4A41-B255-05C7AC6466A0}"/>
   </bookViews>
@@ -1257,11 +1257,11 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="11">
@@ -2133,6 +2133,36 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="lt1">
+                  <a:lumMod val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-ES"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
@@ -3019,6 +3049,36 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="lt1">
+                  <a:lumMod val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-ES"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
@@ -4304,7 +4364,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{F5014612-C4A0-4CF6-8A40-27AEDB09F189}" type="CELLRANGE">
+                    <a:fld id="{5FB01BBD-CC8F-4BFA-82DE-E75A835ED0C3}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4337,7 +4397,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{CEE9638C-D09E-419D-B1DE-4AE7B698505E}" type="CELLRANGE">
+                    <a:fld id="{0193D479-2D69-4FCA-AA36-AB2448444AE8}" type="CELLRANGE">
                       <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4371,7 +4431,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{F0064F89-064F-4068-A3E5-B75D7B2D10D0}" type="CELLRANGE">
+                    <a:fld id="{335ADB76-B767-4F69-81FF-CD98717D9AC3}" type="CELLRANGE">
                       <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4405,7 +4465,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{3E1107B1-9366-4673-8A06-C34E1299323F}" type="CELLRANGE">
+                    <a:fld id="{EEECFD1E-AE76-4DC9-8D00-5D5428CCA9AD}" type="CELLRANGE">
                       <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4439,7 +4499,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{563E76D3-5A64-4DB7-949D-88515440BF4F}" type="CELLRANGE">
+                    <a:fld id="{91A67CD8-7391-4106-913D-824B3C315102}" type="CELLRANGE">
                       <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4473,7 +4533,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{85D16B28-1912-438B-9860-AD9CD9F05B8E}" type="CELLRANGE">
+                    <a:fld id="{20884954-FB44-4038-835A-7A469CF71542}" type="CELLRANGE">
                       <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4507,7 +4567,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{AD7DF104-1A44-4063-B955-C36D5C06E219}" type="CELLRANGE">
+                    <a:fld id="{3E4B359C-9CFA-49A8-BEC9-81586AE3B9EB}" type="CELLRANGE">
                       <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4541,7 +4601,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{4D9F10D5-A17F-497C-859A-F3EBEC459CFD}" type="CELLRANGE">
+                    <a:fld id="{A842D766-4500-4F16-BC7C-9935EF5E1E7F}" type="CELLRANGE">
                       <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4575,7 +4635,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{8643BD52-8E40-4F67-9208-FA2FABA14393}" type="CELLRANGE">
+                    <a:fld id="{AE2B48DD-B870-408F-8EA3-0E785820CC75}" type="CELLRANGE">
                       <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4609,7 +4669,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{361C9932-CF51-4845-8C28-D07D546F1A96}" type="CELLRANGE">
+                    <a:fld id="{34B76F97-CAB7-4714-810F-E32384780AD0}" type="CELLRANGE">
                       <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4643,7 +4703,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{A0708591-975E-4A88-9488-FB4ED06E041E}" type="CELLRANGE">
+                    <a:fld id="{4C2EF430-5B66-4291-8949-FC6AE8912D9C}" type="CELLRANGE">
                       <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4677,7 +4737,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{B2FE0FEB-1565-4F3A-AE3C-3BB08F4129FD}" type="CELLRANGE">
+                    <a:fld id="{C6D8A70E-198D-4167-87D5-A20B8BBEBC20}" type="CELLRANGE">
                       <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -5913,40 +5973,40 @@
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>17770.549500000005</c:v>
+                  <c:v>16826.980500000005</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5031.9583999999995</c:v>
+                  <c:v>4807.3173999999999</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>8898.4</c:v>
+                  <c:v>9136.75</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4296.18</c:v>
+                  <c:v>4458.3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4612.6499999999996</c:v>
+                  <c:v>4744.4399999999996</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>6003.72</c:v>
+                  <c:v>5948.13</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>6633.36</c:v>
+                  <c:v>6872.4</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>7112</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>6694.78</c:v>
+                  <c:v>6633.36</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>8749.2000000000007</c:v>
+                  <c:v>8368.7999999999993</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>8553.6</c:v>
+                  <c:v>8475.84</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>8215.98</c:v>
+                  <c:v>7855.63</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7036,40 +7096,40 @@
                 <c:formatCode>_-* #,##0\ _€_-;\-* #,##0\ _€_-;_-* "-"??\ _€_-;_-@_-</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>5441.6024000000007</c:v>
+                  <c:v>5493.9255000000003</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>4537.3230000000003</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1780.4580000000001</c:v>
+                  <c:v>1797.7440000000001</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3499.0695999999998</c:v>
+                  <c:v>3465.4246999999996</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4201.4111999999996</c:v>
+                  <c:v>4282.9920000000002</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>6630.7074000000002</c:v>
+                  <c:v>6695.0832</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>5404.4549999999999</c:v>
+                  <c:v>5301.5130000000008</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>2536.0816</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>3871.92</c:v>
+                  <c:v>3909.15</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2818.7952</c:v>
+                  <c:v>2791.6914000000002</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1693.2760000000001</c:v>
+                  <c:v>1709.5575000000001</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>3535.5162</c:v>
+                  <c:v>3569.8415999999997</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -8021,40 +8081,40 @@
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>12328.947100000005</c:v>
+                  <c:v>11333.055000000004</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>494.63539999999921</c:v>
+                  <c:v>269.99439999999959</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>7117.9419999999991</c:v>
+                  <c:v>7339.0059999999994</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>797.11040000000048</c:v>
+                  <c:v>992.87530000000061</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>411.23880000000008</c:v>
+                  <c:v>461.44799999999941</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-626.98739999999998</c:v>
+                  <c:v>-746.95319999999992</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1228.9049999999997</c:v>
+                  <c:v>1570.8869999999988</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>4575.9184000000005</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2822.8599999999997</c:v>
+                  <c:v>2724.2099999999996</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>5930.4048000000003</c:v>
+                  <c:v>5577.1085999999996</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>6860.3240000000005</c:v>
+                  <c:v>6766.2825000000003</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>4680.4637999999995</c:v>
+                  <c:v>4285.7884000000004</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -13507,10 +13567,10 @@
       <c r="AR1">
         <v>0</v>
       </c>
-      <c r="AT1" s="128" t="s">
+      <c r="AT1" s="129" t="s">
         <v>13</v>
       </c>
-      <c r="AU1" s="128"/>
+      <c r="AU1" s="129"/>
     </row>
     <row r="2" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A2" s="33">
@@ -13762,31 +13822,31 @@
       </c>
       <c r="AF3" s="93">
         <f ca="1">(RANDBETWEEN($AT$3,$AU$3)*Q3/100)+Q3</f>
-        <v>17770.549500000005</v>
+        <v>16826.980500000005</v>
       </c>
       <c r="AG3" s="93">
         <f t="shared" ref="AG3:AQ3" ca="1" si="0">(RANDBETWEEN($AT$3,$AU$3)*R3/100)+R3</f>
-        <v>5031.9583999999995</v>
+        <v>4807.3173999999999</v>
       </c>
       <c r="AH3" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>8898.4</v>
+        <v>9136.75</v>
       </c>
       <c r="AI3" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>4296.18</v>
+        <v>4458.3</v>
       </c>
       <c r="AJ3" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>4612.6499999999996</v>
+        <v>4744.4399999999996</v>
       </c>
       <c r="AK3" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>6003.72</v>
+        <v>5948.13</v>
       </c>
       <c r="AL3" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>6633.36</v>
+        <v>6872.4</v>
       </c>
       <c r="AM3" s="93">
         <f t="shared" ca="1" si="0"/>
@@ -13794,23 +13854,23 @@
       </c>
       <c r="AN3" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>6694.78</v>
+        <v>6633.36</v>
       </c>
       <c r="AO3" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>8749.2000000000007</v>
+        <v>8368.7999999999993</v>
       </c>
       <c r="AP3" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>8553.6</v>
+        <v>8475.84</v>
       </c>
       <c r="AQ3" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>8215.98</v>
+        <v>7855.63</v>
       </c>
       <c r="AR3" s="63">
         <f ca="1">SUM(AF3:AQ3)</f>
-        <v>92572.377900000007</v>
+        <v>91239.947900000014</v>
       </c>
       <c r="AS3" s="53"/>
       <c r="AT3" s="66">
@@ -13852,31 +13912,31 @@
       <c r="AE4" s="8"/>
       <c r="AF4" s="69">
         <f ca="1">AF3/Q3-1</f>
-        <v>0.13000000000000012</v>
+        <v>7.0000000000000062E-2</v>
       </c>
       <c r="AG4" s="69">
         <f t="shared" ref="AG4:AR4" ca="1" si="1">AG3/R3-1</f>
-        <v>0.11999999999999988</v>
+        <v>7.0000000000000062E-2</v>
       </c>
       <c r="AH4" s="69">
         <f t="shared" ca="1" si="1"/>
-        <v>0.11999999999999988</v>
+        <v>0.14999999999999991</v>
       </c>
       <c r="AI4" s="69">
         <f t="shared" ca="1" si="1"/>
-        <v>6.0000000000000053E-2</v>
+        <v>0.10000000000000009</v>
       </c>
       <c r="AJ4" s="69">
         <f t="shared" ca="1" si="1"/>
-        <v>4.9999999999999822E-2</v>
+        <v>7.9999999999999849E-2</v>
       </c>
       <c r="AK4" s="69">
         <f t="shared" ca="1" si="1"/>
-        <v>8.0000000000000071E-2</v>
+        <v>7.0000000000000062E-2</v>
       </c>
       <c r="AL4" s="69">
         <f t="shared" ca="1" si="1"/>
-        <v>0.10999999999999988</v>
+        <v>0.14999999999999991</v>
       </c>
       <c r="AM4" s="69">
         <f t="shared" ca="1" si="1"/>
@@ -13884,23 +13944,23 @@
       </c>
       <c r="AN4" s="69">
         <f t="shared" ca="1" si="1"/>
-        <v>8.9999999999999858E-2</v>
+        <v>7.9999999999999849E-2</v>
       </c>
       <c r="AO4" s="69">
         <f t="shared" ca="1" si="1"/>
-        <v>0.15000000000000013</v>
+        <v>9.9999999999999867E-2</v>
       </c>
       <c r="AP4" s="69">
         <f t="shared" ca="1" si="1"/>
-        <v>0.10000000000000009</v>
+        <v>9.000000000000008E-2</v>
       </c>
       <c r="AQ4" s="69">
         <f t="shared" ca="1" si="1"/>
-        <v>0.1399999999999999</v>
+        <v>9.000000000000008E-2</v>
       </c>
       <c r="AR4" s="69">
         <f t="shared" ca="1" si="1"/>
-        <v>0.11227485063014275</v>
+        <v>9.6265448983076318E-2</v>
       </c>
       <c r="AS4" s="53"/>
     </row>
@@ -14033,10 +14093,10 @@
         <f t="shared" ref="AR5" si="2">SUM(AF5:AQ5)</f>
         <v>0</v>
       </c>
-      <c r="AT5" s="128" t="s">
+      <c r="AT5" s="129" t="s">
         <v>35</v>
       </c>
-      <c r="AU5" s="128"/>
+      <c r="AU5" s="129"/>
     </row>
     <row r="6" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A6" s="28" t="s">
@@ -15970,7 +16030,7 @@
       </c>
       <c r="AF22" s="51">
         <f ca="1">(RANDBETWEEN($AT$7,$AU$7)*Q22/100)+Q22</f>
-        <v>5441.6024000000007</v>
+        <v>5493.9255000000003</v>
       </c>
       <c r="AG22" s="51">
         <f t="shared" ref="AG22:AQ22" ca="1" si="18">(RANDBETWEEN($AT$7,$AU$7)*R22/100)+R22</f>
@@ -15978,23 +16038,23 @@
       </c>
       <c r="AH22" s="51">
         <f t="shared" ca="1" si="18"/>
-        <v>1780.4580000000001</v>
+        <v>1797.7440000000001</v>
       </c>
       <c r="AI22" s="51">
         <f t="shared" ca="1" si="18"/>
-        <v>3499.0695999999998</v>
+        <v>3465.4246999999996</v>
       </c>
       <c r="AJ22" s="51">
         <f t="shared" ca="1" si="18"/>
-        <v>4201.4111999999996</v>
+        <v>4282.9920000000002</v>
       </c>
       <c r="AK22" s="51">
         <f t="shared" ca="1" si="18"/>
-        <v>6630.7074000000002</v>
+        <v>6695.0832</v>
       </c>
       <c r="AL22" s="51">
         <f t="shared" ca="1" si="18"/>
-        <v>5404.4549999999999</v>
+        <v>5301.5130000000008</v>
       </c>
       <c r="AM22" s="51">
         <f t="shared" ca="1" si="18"/>
@@ -16002,23 +16062,23 @@
       </c>
       <c r="AN22" s="51">
         <f t="shared" ca="1" si="18"/>
-        <v>3871.92</v>
+        <v>3909.15</v>
       </c>
       <c r="AO22" s="51">
         <f t="shared" ca="1" si="18"/>
-        <v>2818.7952</v>
+        <v>2791.6914000000002</v>
       </c>
       <c r="AP22" s="51">
         <f t="shared" ca="1" si="18"/>
-        <v>1693.2760000000001</v>
+        <v>1709.5575000000001</v>
       </c>
       <c r="AQ22" s="51">
         <f t="shared" ca="1" si="18"/>
-        <v>3535.5162</v>
+        <v>3569.8415999999997</v>
       </c>
       <c r="AR22" s="52">
         <f ca="1">SUM(AF22:AQ22)</f>
-        <v>45950.61559999999</v>
+        <v>46090.327500000007</v>
       </c>
     </row>
     <row r="23" spans="1:47" x14ac:dyDescent="0.3">
@@ -16137,31 +16197,31 @@
       </c>
       <c r="AF23" s="6">
         <f t="shared" ref="AF23:AQ23" ca="1" si="21">AF3-AF7-AF12</f>
-        <v>17770.549500000005</v>
+        <v>16826.980500000005</v>
       </c>
       <c r="AG23" s="6">
         <f t="shared" ca="1" si="21"/>
-        <v>5031.9583999999995</v>
+        <v>4807.3173999999999</v>
       </c>
       <c r="AH23" s="6">
         <f t="shared" ca="1" si="21"/>
-        <v>8898.4</v>
+        <v>9136.75</v>
       </c>
       <c r="AI23" s="6">
         <f t="shared" ca="1" si="21"/>
-        <v>4296.18</v>
+        <v>4458.3</v>
       </c>
       <c r="AJ23" s="6">
         <f t="shared" ca="1" si="21"/>
-        <v>4612.6499999999996</v>
+        <v>4744.4399999999996</v>
       </c>
       <c r="AK23" s="6">
         <f t="shared" ca="1" si="21"/>
-        <v>6003.72</v>
+        <v>5948.13</v>
       </c>
       <c r="AL23" s="6">
         <f t="shared" ca="1" si="21"/>
-        <v>6633.36</v>
+        <v>6872.4</v>
       </c>
       <c r="AM23" s="6">
         <f t="shared" ca="1" si="21"/>
@@ -16169,23 +16229,23 @@
       </c>
       <c r="AN23" s="6">
         <f t="shared" ca="1" si="21"/>
-        <v>6694.78</v>
+        <v>6633.36</v>
       </c>
       <c r="AO23" s="6">
         <f t="shared" ca="1" si="21"/>
-        <v>8749.2000000000007</v>
+        <v>8368.7999999999993</v>
       </c>
       <c r="AP23" s="6">
         <f t="shared" ca="1" si="21"/>
-        <v>8553.6</v>
+        <v>8475.84</v>
       </c>
       <c r="AQ23" s="6">
         <f t="shared" ca="1" si="21"/>
-        <v>8215.98</v>
+        <v>7855.63</v>
       </c>
       <c r="AR23" s="7">
         <f ca="1">SUM(AF23:AQ23)</f>
-        <v>92572.377900000007</v>
+        <v>91239.947900000014</v>
       </c>
     </row>
     <row r="24" spans="1:47" x14ac:dyDescent="0.3">
@@ -16534,31 +16594,31 @@
       </c>
       <c r="AF28" s="32">
         <f ca="1">AF3-AF22</f>
-        <v>12328.947100000005</v>
+        <v>11333.055000000004</v>
       </c>
       <c r="AG28" s="32">
         <f t="shared" ref="AG28:AQ28" ca="1" si="25">AG3-AG22</f>
-        <v>494.63539999999921</v>
+        <v>269.99439999999959</v>
       </c>
       <c r="AH28" s="32">
         <f t="shared" ca="1" si="25"/>
-        <v>7117.9419999999991</v>
+        <v>7339.0059999999994</v>
       </c>
       <c r="AI28" s="32">
         <f t="shared" ca="1" si="25"/>
-        <v>797.11040000000048</v>
+        <v>992.87530000000061</v>
       </c>
       <c r="AJ28" s="32">
         <f t="shared" ca="1" si="25"/>
-        <v>411.23880000000008</v>
+        <v>461.44799999999941</v>
       </c>
       <c r="AK28" s="32">
         <f t="shared" ca="1" si="25"/>
-        <v>-626.98739999999998</v>
+        <v>-746.95319999999992</v>
       </c>
       <c r="AL28" s="32">
         <f t="shared" ca="1" si="25"/>
-        <v>1228.9049999999997</v>
+        <v>1570.8869999999988</v>
       </c>
       <c r="AM28" s="32">
         <f t="shared" ca="1" si="25"/>
@@ -16566,23 +16626,23 @@
       </c>
       <c r="AN28" s="32">
         <f t="shared" ca="1" si="25"/>
-        <v>2822.8599999999997</v>
+        <v>2724.2099999999996</v>
       </c>
       <c r="AO28" s="32">
         <f t="shared" ca="1" si="25"/>
-        <v>5930.4048000000003</v>
+        <v>5577.1085999999996</v>
       </c>
       <c r="AP28" s="32">
         <f t="shared" ca="1" si="25"/>
-        <v>6860.3240000000005</v>
+        <v>6766.2825000000003</v>
       </c>
       <c r="AQ28" s="32">
         <f t="shared" ca="1" si="25"/>
-        <v>4680.4637999999995</v>
+        <v>4285.7884000000004</v>
       </c>
       <c r="AR28" s="32">
         <f ca="1">SUM(AF28:AQ28)</f>
-        <v>46621.762300000009</v>
+        <v>45149.6204</v>
       </c>
     </row>
     <row r="29" spans="1:47" x14ac:dyDescent="0.3">
@@ -16745,31 +16805,31 @@
       </c>
       <c r="AF30" s="15">
         <f t="shared" ref="AF30:AQ30" ca="1" si="28">AF28</f>
-        <v>12328.947100000005</v>
+        <v>11333.055000000004</v>
       </c>
       <c r="AG30" s="15">
         <f t="shared" ca="1" si="28"/>
-        <v>494.63539999999921</v>
+        <v>269.99439999999959</v>
       </c>
       <c r="AH30" s="15">
         <f t="shared" ca="1" si="28"/>
-        <v>7117.9419999999991</v>
+        <v>7339.0059999999994</v>
       </c>
       <c r="AI30" s="15">
         <f t="shared" ca="1" si="28"/>
-        <v>797.11040000000048</v>
+        <v>992.87530000000061</v>
       </c>
       <c r="AJ30" s="15">
         <f t="shared" ca="1" si="28"/>
-        <v>411.23880000000008</v>
+        <v>461.44799999999941</v>
       </c>
       <c r="AK30" s="15">
         <f t="shared" ca="1" si="28"/>
-        <v>-626.98739999999998</v>
+        <v>-746.95319999999992</v>
       </c>
       <c r="AL30" s="15">
         <f t="shared" ca="1" si="28"/>
-        <v>1228.9049999999997</v>
+        <v>1570.8869999999988</v>
       </c>
       <c r="AM30" s="15">
         <f t="shared" ca="1" si="28"/>
@@ -16777,23 +16837,23 @@
       </c>
       <c r="AN30" s="15">
         <f t="shared" ca="1" si="28"/>
-        <v>2822.8599999999997</v>
+        <v>2724.2099999999996</v>
       </c>
       <c r="AO30" s="15">
         <f t="shared" ca="1" si="28"/>
-        <v>5930.4048000000003</v>
+        <v>5577.1085999999996</v>
       </c>
       <c r="AP30" s="15">
         <f t="shared" ca="1" si="28"/>
-        <v>6860.3240000000005</v>
+        <v>6766.2825000000003</v>
       </c>
       <c r="AQ30" s="15">
         <f t="shared" ca="1" si="28"/>
-        <v>4680.4637999999995</v>
+        <v>4285.7884000000004</v>
       </c>
       <c r="AR30" s="15">
         <f ca="1">SUM(AF30:AQ30)</f>
-        <v>46621.762300000009</v>
+        <v>45149.6204</v>
       </c>
     </row>
     <row r="31" spans="1:47" x14ac:dyDescent="0.3">
@@ -16904,31 +16964,31 @@
       <c r="AE31" s="10"/>
       <c r="AF31" s="16">
         <f t="shared" ref="AF31:AR31" ca="1" si="31">AF30/AF3</f>
-        <v>0.69378536099854438</v>
+        <v>0.67350497018761035</v>
       </c>
       <c r="AG31" s="16">
         <f t="shared" ca="1" si="31"/>
-        <v>9.8298785617941364E-2</v>
+        <v>5.6163214852424682E-2</v>
       </c>
       <c r="AH31" s="16">
         <f t="shared" ca="1" si="31"/>
-        <v>0.79991256855164972</v>
+        <v>0.80324032068295614</v>
       </c>
       <c r="AI31" s="16">
         <f t="shared" ca="1" si="31"/>
-        <v>0.18553933959936511</v>
+        <v>0.22270266693582769</v>
       </c>
       <c r="AJ31" s="16">
         <f t="shared" ca="1" si="31"/>
-        <v>8.9154564079216958E-2</v>
+        <v>9.7260793686926056E-2</v>
       </c>
       <c r="AK31" s="16">
         <f t="shared" ca="1" si="31"/>
-        <v>-0.10443315144610341</v>
+        <v>-0.12557782025611408</v>
       </c>
       <c r="AL31" s="16">
         <f t="shared" ca="1" si="31"/>
-        <v>0.18526131553239983</v>
+        <v>0.22857909900471435</v>
       </c>
       <c r="AM31" s="16">
         <f t="shared" ca="1" si="31"/>
@@ -16936,23 +16996,23 @@
       </c>
       <c r="AN31" s="16">
         <f t="shared" ca="1" si="31"/>
-        <v>0.42165089816244894</v>
+        <v>0.41068327363508084</v>
       </c>
       <c r="AO31" s="16">
         <f t="shared" ca="1" si="31"/>
-        <v>0.67782252091619799</v>
+        <v>0.66641676225982216</v>
       </c>
       <c r="AP31" s="16">
         <f t="shared" ca="1" si="31"/>
-        <v>0.80203937523381974</v>
+        <v>0.79830229216219284</v>
       </c>
       <c r="AQ31" s="16">
         <f t="shared" ca="1" si="31"/>
-        <v>0.56967809074510889</v>
+        <v>0.54556902501772619</v>
       </c>
       <c r="AR31" s="16">
         <f t="shared" ca="1" si="31"/>
-        <v>0.50362498358163066</v>
+        <v>0.49484487265911725</v>
       </c>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.3">
@@ -17100,60 +17160,60 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:28" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="129" t="str">
+      <c r="A2" s="128" t="str">
         <f>CONCATENATE("Ventas totales", " ", I8)</f>
         <v>Ventas totales Mayo</v>
       </c>
-      <c r="B2" s="129"/>
-      <c r="C2" s="129"/>
-      <c r="D2" s="129"/>
-      <c r="E2" s="129"/>
-      <c r="F2" s="129"/>
-      <c r="U2" s="129" t="str">
+      <c r="B2" s="128"/>
+      <c r="C2" s="128"/>
+      <c r="D2" s="128"/>
+      <c r="E2" s="128"/>
+      <c r="F2" s="128"/>
+      <c r="U2" s="128" t="str">
         <f>CONCATENATE("Ventas acumuladas")</f>
         <v>Ventas acumuladas</v>
       </c>
-      <c r="V2" s="129"/>
-      <c r="W2" s="129"/>
-      <c r="X2" s="129"/>
-      <c r="Y2" s="129"/>
-      <c r="Z2" s="129"/>
-      <c r="AA2" s="129"/>
-      <c r="AB2" s="129"/>
+      <c r="V2" s="128"/>
+      <c r="W2" s="128"/>
+      <c r="X2" s="128"/>
+      <c r="Y2" s="128"/>
+      <c r="Z2" s="128"/>
+      <c r="AA2" s="128"/>
+      <c r="AB2" s="128"/>
     </row>
     <row r="3" spans="1:28" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="129"/>
-      <c r="B3" s="129"/>
-      <c r="C3" s="129"/>
-      <c r="D3" s="129"/>
-      <c r="E3" s="129"/>
-      <c r="F3" s="129"/>
+      <c r="A3" s="128"/>
+      <c r="B3" s="128"/>
+      <c r="C3" s="128"/>
+      <c r="D3" s="128"/>
+      <c r="E3" s="128"/>
+      <c r="F3" s="128"/>
       <c r="G3" s="98"/>
-      <c r="U3" s="129"/>
-      <c r="V3" s="129"/>
-      <c r="W3" s="129"/>
-      <c r="X3" s="129"/>
-      <c r="Y3" s="129"/>
-      <c r="Z3" s="129"/>
-      <c r="AA3" s="129"/>
-      <c r="AB3" s="129"/>
+      <c r="U3" s="128"/>
+      <c r="V3" s="128"/>
+      <c r="W3" s="128"/>
+      <c r="X3" s="128"/>
+      <c r="Y3" s="128"/>
+      <c r="Z3" s="128"/>
+      <c r="AA3" s="128"/>
+      <c r="AB3" s="128"/>
     </row>
     <row r="4" spans="1:28" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="129"/>
-      <c r="B4" s="129"/>
-      <c r="C4" s="129"/>
-      <c r="D4" s="129"/>
-      <c r="E4" s="129"/>
-      <c r="F4" s="129"/>
+      <c r="A4" s="128"/>
+      <c r="B4" s="128"/>
+      <c r="C4" s="128"/>
+      <c r="D4" s="128"/>
+      <c r="E4" s="128"/>
+      <c r="F4" s="128"/>
       <c r="G4" s="98"/>
-      <c r="U4" s="129"/>
-      <c r="V4" s="129"/>
-      <c r="W4" s="129"/>
-      <c r="X4" s="129"/>
-      <c r="Y4" s="129"/>
-      <c r="Z4" s="129"/>
-      <c r="AA4" s="129"/>
-      <c r="AB4" s="129"/>
+      <c r="U4" s="128"/>
+      <c r="V4" s="128"/>
+      <c r="W4" s="128"/>
+      <c r="X4" s="128"/>
+      <c r="Y4" s="128"/>
+      <c r="Z4" s="128"/>
+      <c r="AA4" s="128"/>
+      <c r="AB4" s="128"/>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="N5" s="126"/>
@@ -17235,19 +17295,19 @@
       </c>
       <c r="Q9" s="114">
         <f ca="1">VLOOKUP(H9,'Cta Resultados'!$AE$3:$AR$30,MATCH('Mi dashboard'!$I$8,'Cta Resultados'!$AE$2:$AR$2,0),0)</f>
-        <v>4612.6499999999996</v>
+        <v>4744.4399999999996</v>
       </c>
       <c r="R9" s="111">
         <f ca="1">IFERROR(I9/Q9-1,"")</f>
-        <v>-0.12132938766218981</v>
+        <v>-0.14573690467157341</v>
       </c>
       <c r="S9" s="122">
         <f ca="1">SUMPRODUCT('Cta Resultados'!AF3:AQ3,'Cta Resultados'!AF1:AQ1)</f>
-        <v>60358.817900000009</v>
+        <v>59906.317900000009</v>
       </c>
       <c r="T9" s="113">
         <f ca="1">IFERROR(I9/S9-1,"")</f>
-        <v>-0.93285156765802069</v>
+        <v>-0.93234436463336701</v>
       </c>
     </row>
     <row r="10" spans="1:28" ht="21" x14ac:dyDescent="0.4">
@@ -17475,19 +17535,19 @@
       <c r="P17" s="109"/>
       <c r="Q17" s="117">
         <f ca="1">VLOOKUP('Cta Resultados'!AE30,'Cta Resultados'!$AE$3:$AR$30,MATCH('Mi dashboard'!$I$8,'Cta Resultados'!$AE$2:$AR$2,0),0)</f>
-        <v>411.23880000000008</v>
+        <v>461.44799999999941</v>
       </c>
       <c r="R17" s="119">
         <f ca="1">IFERROR(I17/Q17-1,"")</f>
-        <v>0.6742340460092775</v>
+        <v>0.49206411123247062</v>
       </c>
       <c r="S17" s="123">
         <f ca="1">SUMPRODUCT('Cta Resultados'!AF30:AQ30,'Cta Resultados'!AF1:AQ1)</f>
-        <v>26327.709700000007</v>
+        <v>25796.230900000002</v>
       </c>
       <c r="T17" s="119">
         <f ca="1">IFERROR(I17/S17-1,"")</f>
-        <v>-0.97384846582382367</v>
+        <v>-0.97330966672344366</v>
       </c>
       <c r="U17" s="109"/>
     </row>

</xml_diff>